<commit_message>
Improve metadata and add validations
</commit_message>
<xml_diff>
--- a/ro-crate-validation.xlsx
+++ b/ro-crate-validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alvinsw/uqslc/codes/corpus-tools-cooee/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6AB865-1257-AA40-B70D-4AE4ABE89ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699280FE-78C4-6E4C-A659-C54E7142A8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1740" yWindow="1680" windowWidth="27240" windowHeight="16420" activeTab="1" xr2:uid="{756E4AC4-F825-4F44-B76C-9C1C961306D6}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="types" sheetId="1" r:id="rId1"/>
     <sheet name="properties" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -487,7 +487,7 @@
         <v>9</v>
       </c>
       <c r="C4">
-        <v>1358</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -542,7 +542,7 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>2713</v>
+        <v>2709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix the type of entity that is a specialization of another
</commit_message>
<xml_diff>
--- a/ro-crate-validation.xlsx
+++ b/ro-crate-validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cjhaseloff/Documents/GitHub/LDaCA/corpus-tools-cooee/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alvinsw/uqslc/codes/corpus-tools-cooee/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0B1816-71EA-4E41-9C88-E09047F684EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF5034D-1934-6049-9522-9F2A10FCD8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="1100" windowWidth="27240" windowHeight="16420" activeTab="1" xr2:uid="{756E4AC4-F825-4F44-B76C-9C1C961306D6}"/>
+    <workbookView xWindow="1160" yWindow="1100" windowWidth="27240" windowHeight="16420" xr2:uid="{756E4AC4-F825-4F44-B76C-9C1C961306D6}"/>
   </bookViews>
   <sheets>
     <sheet name="types" sheetId="1" r:id="rId1"/>
@@ -459,7 +459,7 @@
         <v>2</v>
       </c>
       <c r="C2">
-        <v>2713</v>
+        <v>2714</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>